<commit_message>
fix: en-tête HTML complet + Mongré retiré des clients probables
Notre-Dame de Mongré entre au 7e rang du top 25. Le script et le fichier
CRM sont alignés sur la page, et les liens de téléchargement sont gardés.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/edai_prive_academie_lyon.xlsx
+++ b/edai_prive_academie_lyon.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Top 25'!$A$1:$P$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tous les comptes'!$A$1:$P$127</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Clients probables'!$A$1:$P$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Clients probables'!$A$1:$P$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Détail par établissement'!$A$1:$H$175</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,14 +468,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Top 25 : 34 827 élèves · 208 962 €/an sur 1 matière</t>
+          <t>Top 25 : 36 017 élèves · 216 102 €/an sur 1 matière</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Clients probables (réseau CSND, à vérifier) : NOTRE DAME DE MONGRE, NOTRE DAME DE BEL AIR, NOTRE DAME, NOTRE DAME, NOTRE DAME DU MAS, NOTRE DAME</t>
+          <t>Clients probables (réseau CSND, à vérifier) : NOTRE DAME DE BEL AIR, NOTRE DAME, NOTRE DAME, NOTRE DAME DU MAS, NOTRE DAME</t>
         </is>
       </c>
     </row>
@@ -971,12 +971,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SAINT LOUIS-SAINT BRUNO</t>
+          <t>NOTRE DAME DE MONGRE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LYON</t>
+          <t>VILLEFRANCHE-SUR-SAONE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -990,22 +990,22 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1410</v>
+        <v>1789</v>
       </c>
       <c r="G8" t="n">
-        <v>859</v>
+        <v>1115</v>
       </c>
       <c r="H8" t="n">
-        <v>551</v>
+        <v>674</v>
       </c>
       <c r="I8" t="n">
-        <v>8460</v>
+        <v>10734</v>
       </c>
       <c r="J8" t="n">
-        <v>25380</v>
+        <v>32202</v>
       </c>
       <c r="K8" t="n">
-        <v>3.1</v>
+        <v>28.8</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1014,16 +1014,16 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>13748</v>
+        <v>15430</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>https://www.slsb.fr/college/</t>
+          <t>https://www.mongre.org/</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0692929J, 0690563M</t>
+          <t>0692944A, 0690552A</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SAINT MARC</t>
+          <t>SAINT LOUIS-SAINT BRUNO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1052,22 +1052,22 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1375</v>
+        <v>1410</v>
       </c>
       <c r="G9" t="n">
-        <v>525</v>
+        <v>859</v>
       </c>
       <c r="H9" t="n">
-        <v>850</v>
+        <v>551</v>
       </c>
       <c r="I9" t="n">
-        <v>8250</v>
+        <v>8460</v>
       </c>
       <c r="J9" t="n">
-        <v>24750</v>
+        <v>25380</v>
       </c>
       <c r="K9" t="n">
-        <v>1.7</v>
+        <v>3.1</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1076,16 +1076,16 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>13406</v>
+        <v>13748</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>https://www.collegesaintmarc.org/</t>
+          <t>https://www.slsb.fr/college/</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0692931L, 0690641X, 0690571W</t>
+          <t>0692929J, 0690563M</t>
         </is>
       </c>
     </row>
@@ -1095,17 +1095,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SAINTE MARIE LA GRAND'GRANGE</t>
+          <t>SAINT MARC</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SAINT-CHAMOND</t>
+          <t>LYON</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1114,22 +1114,22 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1538</v>
+        <v>1375</v>
       </c>
       <c r="G10" t="n">
-        <v>1152</v>
+        <v>525</v>
       </c>
       <c r="H10" t="n">
-        <v>386</v>
+        <v>850</v>
       </c>
       <c r="I10" t="n">
-        <v>9228</v>
+        <v>8250</v>
       </c>
       <c r="J10" t="n">
-        <v>27684</v>
+        <v>24750</v>
       </c>
       <c r="K10" t="n">
-        <v>39.7</v>
+        <v>1.7</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1138,16 +1138,16 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>13265</v>
+        <v>13406</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>https://ismgg.fr/lycee-professionnel/</t>
+          <t>https://www.collegesaintmarc.org/</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>0420996E, 0421799C, 0421022H</t>
+          <t>0692931L, 0690641X, 0690571W</t>
         </is>
       </c>
     </row>
@@ -1157,17 +1157,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CHEVREUL LESTONNAC</t>
+          <t>SAINTE MARIE LA GRAND'GRANGE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LYON</t>
+          <t>SAINT-CHAMOND</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1176,22 +1176,22 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1356</v>
+        <v>1538</v>
       </c>
       <c r="G11" t="n">
-        <v>481</v>
+        <v>1152</v>
       </c>
       <c r="H11" t="n">
-        <v>875</v>
+        <v>386</v>
       </c>
       <c r="I11" t="n">
-        <v>8136</v>
+        <v>9228</v>
       </c>
       <c r="J11" t="n">
-        <v>24408</v>
+        <v>27684</v>
       </c>
       <c r="K11" t="n">
-        <v>1.2</v>
+        <v>39.7</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -1200,16 +1200,16 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>13221</v>
+        <v>13265</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>http://www.chevreullestonnac.fr/</t>
+          <t>https://ismgg.fr/lycee-professionnel/</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>0692922B, 0690574Z</t>
+          <t>0420996E, 0421799C, 0421022H</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LA FAVORITE SAINTE THERESE</t>
+          <t>CHEVREUL LESTONNAC</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1238,22 +1238,22 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1345</v>
+        <v>1356</v>
       </c>
       <c r="G12" t="n">
-        <v>728</v>
+        <v>481</v>
       </c>
       <c r="H12" t="n">
-        <v>617</v>
+        <v>875</v>
       </c>
       <c r="I12" t="n">
-        <v>8070</v>
+        <v>8136</v>
       </c>
       <c r="J12" t="n">
-        <v>24210</v>
+        <v>24408</v>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
+        <v>1.2</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1262,16 +1262,16 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>13114</v>
+        <v>13221</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>https://www.la-favorite.org/college/</t>
+          <t>http://www.chevreullestonnac.fr/</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>0692937T, 0690520R</t>
+          <t>0692922B, 0690574Z</t>
         </is>
       </c>
     </row>
@@ -1281,12 +1281,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SAINT JOSEPH</t>
+          <t>LA FAVORITE SAINTE THERESE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TASSIN-LA-DEMI-LUNE</t>
+          <t>LYON</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1303,10 +1303,10 @@
         <v>1345</v>
       </c>
       <c r="G13" t="n">
-        <v>843</v>
+        <v>728</v>
       </c>
       <c r="H13" t="n">
-        <v>502</v>
+        <v>617</v>
       </c>
       <c r="I13" t="n">
         <v>8070</v>
@@ -1315,7 +1315,7 @@
         <v>24210</v>
       </c>
       <c r="K13" t="n">
-        <v>6.8</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>https://www.stjosephtassin.org/</t>
+          <t>https://www.la-favorite.org/college/</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>0692943Z, 0690550Y</t>
+          <t>0692937T, 0690520R</t>
         </is>
       </c>
     </row>
@@ -1343,12 +1343,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IMMACULEE CONCEPTION</t>
+          <t>SAINT JOSEPH</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>VILLEURBANNE</t>
+          <t>TASSIN-LA-DEMI-LUNE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1362,22 +1362,22 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1293</v>
+        <v>1345</v>
       </c>
       <c r="G14" t="n">
-        <v>788</v>
+        <v>843</v>
       </c>
       <c r="H14" t="n">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="I14" t="n">
-        <v>7758</v>
+        <v>8070</v>
       </c>
       <c r="J14" t="n">
-        <v>23274</v>
+        <v>24210</v>
       </c>
       <c r="K14" t="n">
-        <v>3.8</v>
+        <v>6.8</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1386,16 +1386,16 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>12607</v>
+        <v>13114</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>https://college-immac.immaculee.net/</t>
+          <t>https://www.stjosephtassin.org/</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>0692945B, 0690554C</t>
+          <t>0692943Z, 0690550Y</t>
         </is>
       </c>
     </row>
@@ -1405,12 +1405,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NOTRE DAME DES MINIMES</t>
+          <t>IMMACULEE CONCEPTION</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LYON</t>
+          <t>VILLEURBANNE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1424,22 +1424,22 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1270</v>
+        <v>1293</v>
       </c>
       <c r="G15" t="n">
-        <v>641</v>
+        <v>788</v>
       </c>
       <c r="H15" t="n">
-        <v>629</v>
+        <v>505</v>
       </c>
       <c r="I15" t="n">
-        <v>7620</v>
+        <v>7758</v>
       </c>
       <c r="J15" t="n">
-        <v>22860</v>
+        <v>23274</v>
       </c>
       <c r="K15" t="n">
-        <v>4.4</v>
+        <v>3.8</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>12382</v>
+        <v>12607</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>https://www.lesminimes-lyon.org/college/presentation/</t>
+          <t>https://college-immac.immaculee.net/</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0692936S, 0690519P</t>
+          <t>0692945B, 0690554C</t>
         </is>
       </c>
     </row>
@@ -1467,17 +1467,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EXTERNAT SAINT MICHEL</t>
+          <t>NOTRE DAME DES MINIMES</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SAINT-ETIENNE</t>
+          <t>LYON</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1486,22 +1486,22 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1287</v>
+        <v>1270</v>
       </c>
       <c r="G16" t="n">
-        <v>739</v>
+        <v>641</v>
       </c>
       <c r="H16" t="n">
-        <v>548</v>
+        <v>629</v>
       </c>
       <c r="I16" t="n">
-        <v>7722</v>
+        <v>7620</v>
       </c>
       <c r="J16" t="n">
-        <v>23166</v>
+        <v>22860</v>
       </c>
       <c r="K16" t="n">
-        <v>49.5</v>
+        <v>4.4</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -1510,16 +1510,16 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>11100</v>
+        <v>12382</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>https://www.saint-michel-enseignement.com/</t>
+          <t>https://www.lesminimes-lyon.org/college/presentation/</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>0421804H, 0421021G</t>
+          <t>0692936S, 0690519P</t>
         </is>
       </c>
     </row>
@@ -1529,17 +1529,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ASSOMPTION BELLEVUE</t>
+          <t>EXTERNAT SAINT MICHEL</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LA MULATIERE</t>
+          <t>SAINT-ETIENNE</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1548,22 +1548,22 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1107</v>
+        <v>1287</v>
       </c>
       <c r="G17" t="n">
-        <v>480</v>
+        <v>739</v>
       </c>
       <c r="H17" t="n">
-        <v>627</v>
+        <v>548</v>
       </c>
       <c r="I17" t="n">
-        <v>6642</v>
+        <v>7722</v>
       </c>
       <c r="J17" t="n">
-        <v>19926</v>
+        <v>23166</v>
       </c>
       <c r="K17" t="n">
-        <v>2.9</v>
+        <v>49.5</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
@@ -1572,16 +1572,16 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>10793</v>
+        <v>11100</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>https://www.assomption-lyon.org/</t>
+          <t>https://www.saint-michel-enseignement.com/</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0692923C, 0690539L</t>
+          <t>0421804H, 0421021G</t>
         </is>
       </c>
     </row>
@@ -1591,17 +1591,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SAINT PAUL</t>
+          <t>ASSOMPTION BELLEVUE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SAINT-ETIENNE</t>
+          <t>LA MULATIERE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1610,22 +1610,22 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1187</v>
+        <v>1107</v>
       </c>
       <c r="G18" t="n">
-        <v>673</v>
+        <v>480</v>
       </c>
       <c r="H18" t="n">
-        <v>514</v>
+        <v>627</v>
       </c>
       <c r="I18" t="n">
-        <v>7122</v>
+        <v>6642</v>
       </c>
       <c r="J18" t="n">
-        <v>21366</v>
+        <v>19926</v>
       </c>
       <c r="K18" t="n">
-        <v>49.6</v>
+        <v>2.9</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -1634,16 +1634,16 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>10238</v>
+        <v>10793</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>https://www.institutionsaintpaul.org</t>
+          <t>https://www.assomption-lyon.org/</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>0421801E, 0421035X</t>
+          <t>0692923C, 0690539L</t>
         </is>
       </c>
     </row>
@@ -1653,17 +1653,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SAINT PIERRE</t>
+          <t>SAINT PAUL</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BOURG-EN-BRESSE</t>
+          <t>SAINT-ETIENNE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1672,22 +1672,22 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1246</v>
+        <v>1187</v>
       </c>
       <c r="G19" t="n">
-        <v>807</v>
+        <v>673</v>
       </c>
       <c r="H19" t="n">
-        <v>439</v>
+        <v>514</v>
       </c>
       <c r="I19" t="n">
-        <v>7476</v>
+        <v>7122</v>
       </c>
       <c r="J19" t="n">
-        <v>22428</v>
+        <v>21366</v>
       </c>
       <c r="K19" t="n">
-        <v>58.4</v>
+        <v>49.6</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1696,16 +1696,16 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>9345</v>
+        <v>10238</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>https://www.college-saintpierre.eu/</t>
+          <t>https://www.institutionsaintpaul.org</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0010082J, 0010070W</t>
+          <t>0421801E, 0421035X</t>
         </is>
       </c>
     </row>
@@ -1715,17 +1715,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CHAMPAGNAT</t>
+          <t>SAINT PIERRE</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SAINT-SYMPHORIEN-SUR-COISE</t>
+          <t>BOURG-EN-BRESSE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1734,22 +1734,22 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1005</v>
+        <v>1246</v>
       </c>
       <c r="G20" t="n">
-        <v>430</v>
+        <v>807</v>
       </c>
       <c r="H20" t="n">
-        <v>575</v>
+        <v>439</v>
       </c>
       <c r="I20" t="n">
-        <v>6030</v>
+        <v>7476</v>
       </c>
       <c r="J20" t="n">
-        <v>18090</v>
+        <v>22428</v>
       </c>
       <c r="K20" t="n">
-        <v>33.2</v>
+        <v>58.4</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1758,16 +1758,16 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>8668</v>
+        <v>9345</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>http://www.champagnat-stsymphorien.eu/index.php</t>
+          <t>https://www.college-saintpierre.eu/</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0692925E, 0691654Y</t>
+          <t>0010082J, 0010070W</t>
         </is>
       </c>
     </row>
@@ -1777,12 +1777,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SAINT CHARLES</t>
+          <t>CHAMPAGNAT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>RILLIEUX-LA-PAPE</t>
+          <t>SAINT-SYMPHORIEN-SUR-COISE</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1796,22 +1796,22 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>864</v>
+        <v>1005</v>
       </c>
       <c r="G21" t="n">
-        <v>628</v>
+        <v>430</v>
       </c>
       <c r="H21" t="n">
-        <v>236</v>
+        <v>575</v>
       </c>
       <c r="I21" t="n">
-        <v>5184</v>
+        <v>6030</v>
       </c>
       <c r="J21" t="n">
-        <v>15552</v>
+        <v>18090</v>
       </c>
       <c r="K21" t="n">
-        <v>8.9</v>
+        <v>33.2</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -1820,16 +1820,16 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>8424</v>
+        <v>8668</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>https://st-charles.eu/</t>
+          <t>http://www.champagnat-stsymphorien.eu/index.php</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>0691680B, 0691651V, 0694197M</t>
+          <t>0692925E, 0691654Y</t>
         </is>
       </c>
     </row>
@@ -1839,17 +1839,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SAINT PAUL</t>
+          <t>SAINT CHARLES</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ROANNE</t>
+          <t>RILLIEUX-LA-PAPE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1858,22 +1858,22 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>927</v>
+        <v>864</v>
       </c>
       <c r="G22" t="n">
-        <v>657</v>
+        <v>628</v>
       </c>
       <c r="H22" t="n">
-        <v>270</v>
+        <v>236</v>
       </c>
       <c r="I22" t="n">
-        <v>5562</v>
+        <v>5184</v>
       </c>
       <c r="J22" t="n">
-        <v>16686</v>
+        <v>15552</v>
       </c>
       <c r="K22" t="n">
-        <v>68</v>
+        <v>8.9</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -1882,16 +1882,16 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>6952</v>
+        <v>8424</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>https://saint-paul-roanne.cybercolleges42.fr/</t>
+          <t>https://st-charles.eu/</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>0421797A, 0421023J</t>
+          <t>0691680B, 0691651V, 0694197M</t>
         </is>
       </c>
     </row>
@@ -1901,12 +1901,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TEZENAS DU MONTCEL</t>
+          <t>SAINT PAUL</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SAINT-ETIENNE</t>
+          <t>ROANNE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1920,22 +1920,22 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>803</v>
+        <v>927</v>
       </c>
       <c r="G23" t="n">
-        <v>495</v>
+        <v>657</v>
       </c>
       <c r="H23" t="n">
-        <v>308</v>
+        <v>270</v>
       </c>
       <c r="I23" t="n">
-        <v>4818</v>
+        <v>5562</v>
       </c>
       <c r="J23" t="n">
-        <v>14454</v>
+        <v>16686</v>
       </c>
       <c r="K23" t="n">
-        <v>49.1</v>
+        <v>68</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -1944,16 +1944,16 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>6926</v>
+        <v>6952</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>https://tezenas.org</t>
+          <t>https://saint-paul-roanne.cybercolleges42.fr/</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>0421741P, 0421742R, 0420979L</t>
+          <t>0421797A, 0421023J</t>
         </is>
       </c>
     </row>
@@ -1963,17 +1963,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SAINT JOSEPH</t>
+          <t>TEZENAS DU MONTCEL</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SAINT-DIDIER-SUR-CHALARONNE</t>
+          <t>SAINT-ETIENNE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1982,22 +1982,22 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>777</v>
+        <v>803</v>
       </c>
       <c r="G24" t="n">
-        <v>557</v>
+        <v>495</v>
       </c>
       <c r="H24" t="n">
-        <v>220</v>
+        <v>308</v>
       </c>
       <c r="I24" t="n">
-        <v>4662</v>
+        <v>4818</v>
       </c>
       <c r="J24" t="n">
-        <v>13986</v>
+        <v>14454</v>
       </c>
       <c r="K24" t="n">
-        <v>47.8</v>
+        <v>49.1</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2006,16 +2006,16 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>6702</v>
+        <v>6926</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>http://www.st-joseph01.fr/</t>
+          <t>https://tezenas.org</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>0010095Y, 0011431A</t>
+          <t>0421741P, 0421742R, 0420979L</t>
         </is>
       </c>
     </row>
@@ -2025,59 +2025,59 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PIERRE TERMIER-SITE MONPLAISIR</t>
+          <t>SAINT JOSEPH</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LYON</t>
+          <t>SAINT-DIDIER-SUR-CHALARONNE</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Collège</t>
+          <t>Collège + Lycée GT</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>849</v>
+        <v>777</v>
       </c>
       <c r="G25" t="n">
-        <v>849</v>
+        <v>557</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="I25" t="n">
-        <v>5094</v>
+        <v>4662</v>
       </c>
       <c r="J25" t="n">
-        <v>15282</v>
+        <v>13986</v>
       </c>
       <c r="K25" t="n">
-        <v>2.4</v>
+        <v>47.8</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>6622</v>
+        <v>6702</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>http://www.etablissement-pierretermier.com</t>
+          <t>http://www.st-joseph01.fr/</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>0692940W</t>
+          <t>0010095Y, 0011431A</t>
         </is>
       </c>
     </row>
@@ -2087,59 +2087,59 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SAINT JOSEPH</t>
+          <t>PIERRE TERMIER-SITE MONPLAISIR</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MIRIBEL</t>
+          <t>LYON</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Collège + Lycée GT</t>
+          <t>Collège</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>599</v>
+        <v>849</v>
       </c>
       <c r="G26" t="n">
-        <v>336</v>
+        <v>849</v>
       </c>
       <c r="H26" t="n">
-        <v>263</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>3594</v>
+        <v>5094</v>
       </c>
       <c r="J26" t="n">
-        <v>10782</v>
+        <v>15282</v>
       </c>
       <c r="K26" t="n">
-        <v>11.9</v>
+        <v>2.4</v>
       </c>
       <c r="L26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>5840</v>
+        <v>6622</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>https://www.saintjoseph01.fr/</t>
+          <t>http://www.etablissement-pierretermier.com</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>0011151W, 0010075B</t>
+          <t>0692940W</t>
         </is>
       </c>
     </row>
@@ -2636,12 +2636,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SAINT LOUIS-SAINT BRUNO</t>
+          <t>NOTRE DAME DE MONGRE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LYON</t>
+          <t>VILLEFRANCHE-SUR-SAONE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2655,22 +2655,22 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1410</v>
+        <v>1789</v>
       </c>
       <c r="G8" t="n">
-        <v>859</v>
+        <v>1115</v>
       </c>
       <c r="H8" t="n">
-        <v>551</v>
+        <v>674</v>
       </c>
       <c r="I8" t="n">
-        <v>8460</v>
+        <v>10734</v>
       </c>
       <c r="J8" t="n">
-        <v>25380</v>
+        <v>32202</v>
       </c>
       <c r="K8" t="n">
-        <v>3.1</v>
+        <v>28.8</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -2679,16 +2679,16 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>13748</v>
+        <v>15430</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>https://www.slsb.fr/college/</t>
+          <t>https://www.mongre.org/</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0692929J, 0690563M</t>
+          <t>0692944A, 0690552A</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SAINT MARC</t>
+          <t>SAINT LOUIS-SAINT BRUNO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2717,22 +2717,22 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1375</v>
+        <v>1410</v>
       </c>
       <c r="G9" t="n">
-        <v>525</v>
+        <v>859</v>
       </c>
       <c r="H9" t="n">
-        <v>850</v>
+        <v>551</v>
       </c>
       <c r="I9" t="n">
-        <v>8250</v>
+        <v>8460</v>
       </c>
       <c r="J9" t="n">
-        <v>24750</v>
+        <v>25380</v>
       </c>
       <c r="K9" t="n">
-        <v>1.7</v>
+        <v>3.1</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -2741,16 +2741,16 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>13406</v>
+        <v>13748</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>https://www.collegesaintmarc.org/</t>
+          <t>https://www.slsb.fr/college/</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0692931L, 0690641X, 0690571W</t>
+          <t>0692929J, 0690563M</t>
         </is>
       </c>
     </row>
@@ -2760,17 +2760,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SAINTE MARIE LA GRAND'GRANGE</t>
+          <t>SAINT MARC</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SAINT-CHAMOND</t>
+          <t>LYON</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -2779,22 +2779,22 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1538</v>
+        <v>1375</v>
       </c>
       <c r="G10" t="n">
-        <v>1152</v>
+        <v>525</v>
       </c>
       <c r="H10" t="n">
-        <v>386</v>
+        <v>850</v>
       </c>
       <c r="I10" t="n">
-        <v>9228</v>
+        <v>8250</v>
       </c>
       <c r="J10" t="n">
-        <v>27684</v>
+        <v>24750</v>
       </c>
       <c r="K10" t="n">
-        <v>39.7</v>
+        <v>1.7</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -2803,16 +2803,16 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>13265</v>
+        <v>13406</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>https://ismgg.fr/lycee-professionnel/</t>
+          <t>https://www.collegesaintmarc.org/</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>0420996E, 0421799C, 0421022H</t>
+          <t>0692931L, 0690641X, 0690571W</t>
         </is>
       </c>
     </row>
@@ -2822,17 +2822,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CHEVREUL LESTONNAC</t>
+          <t>SAINTE MARIE LA GRAND'GRANGE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LYON</t>
+          <t>SAINT-CHAMOND</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2841,22 +2841,22 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1356</v>
+        <v>1538</v>
       </c>
       <c r="G11" t="n">
-        <v>481</v>
+        <v>1152</v>
       </c>
       <c r="H11" t="n">
-        <v>875</v>
+        <v>386</v>
       </c>
       <c r="I11" t="n">
-        <v>8136</v>
+        <v>9228</v>
       </c>
       <c r="J11" t="n">
-        <v>24408</v>
+        <v>27684</v>
       </c>
       <c r="K11" t="n">
-        <v>1.2</v>
+        <v>39.7</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -2865,16 +2865,16 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>13221</v>
+        <v>13265</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>http://www.chevreullestonnac.fr/</t>
+          <t>https://ismgg.fr/lycee-professionnel/</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>0692922B, 0690574Z</t>
+          <t>0420996E, 0421799C, 0421022H</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LA FAVORITE SAINTE THERESE</t>
+          <t>CHEVREUL LESTONNAC</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2903,22 +2903,22 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1345</v>
+        <v>1356</v>
       </c>
       <c r="G12" t="n">
-        <v>728</v>
+        <v>481</v>
       </c>
       <c r="H12" t="n">
-        <v>617</v>
+        <v>875</v>
       </c>
       <c r="I12" t="n">
-        <v>8070</v>
+        <v>8136</v>
       </c>
       <c r="J12" t="n">
-        <v>24210</v>
+        <v>24408</v>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
+        <v>1.2</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -2927,16 +2927,16 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>13114</v>
+        <v>13221</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>https://www.la-favorite.org/college/</t>
+          <t>http://www.chevreullestonnac.fr/</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>0692937T, 0690520R</t>
+          <t>0692922B, 0690574Z</t>
         </is>
       </c>
     </row>
@@ -2946,12 +2946,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SAINT JOSEPH</t>
+          <t>LA FAVORITE SAINTE THERESE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TASSIN-LA-DEMI-LUNE</t>
+          <t>LYON</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2968,10 +2968,10 @@
         <v>1345</v>
       </c>
       <c r="G13" t="n">
-        <v>843</v>
+        <v>728</v>
       </c>
       <c r="H13" t="n">
-        <v>502</v>
+        <v>617</v>
       </c>
       <c r="I13" t="n">
         <v>8070</v>
@@ -2980,7 +2980,7 @@
         <v>24210</v>
       </c>
       <c r="K13" t="n">
-        <v>6.8</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -2993,12 +2993,12 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>https://www.stjosephtassin.org/</t>
+          <t>https://www.la-favorite.org/college/</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>0692943Z, 0690550Y</t>
+          <t>0692937T, 0690520R</t>
         </is>
       </c>
     </row>
@@ -3008,12 +3008,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IMMACULEE CONCEPTION</t>
+          <t>SAINT JOSEPH</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>VILLEURBANNE</t>
+          <t>TASSIN-LA-DEMI-LUNE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -3027,22 +3027,22 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1293</v>
+        <v>1345</v>
       </c>
       <c r="G14" t="n">
-        <v>788</v>
+        <v>843</v>
       </c>
       <c r="H14" t="n">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="I14" t="n">
-        <v>7758</v>
+        <v>8070</v>
       </c>
       <c r="J14" t="n">
-        <v>23274</v>
+        <v>24210</v>
       </c>
       <c r="K14" t="n">
-        <v>3.8</v>
+        <v>6.8</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -3051,16 +3051,16 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>12607</v>
+        <v>13114</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>https://college-immac.immaculee.net/</t>
+          <t>https://www.stjosephtassin.org/</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>0692945B, 0690554C</t>
+          <t>0692943Z, 0690550Y</t>
         </is>
       </c>
     </row>
@@ -3070,12 +3070,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NOTRE DAME DES MINIMES</t>
+          <t>IMMACULEE CONCEPTION</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LYON</t>
+          <t>VILLEURBANNE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -3089,22 +3089,22 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1270</v>
+        <v>1293</v>
       </c>
       <c r="G15" t="n">
-        <v>641</v>
+        <v>788</v>
       </c>
       <c r="H15" t="n">
-        <v>629</v>
+        <v>505</v>
       </c>
       <c r="I15" t="n">
-        <v>7620</v>
+        <v>7758</v>
       </c>
       <c r="J15" t="n">
-        <v>22860</v>
+        <v>23274</v>
       </c>
       <c r="K15" t="n">
-        <v>4.4</v>
+        <v>3.8</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -3113,16 +3113,16 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>12382</v>
+        <v>12607</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>https://www.lesminimes-lyon.org/college/presentation/</t>
+          <t>https://college-immac.immaculee.net/</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0692936S, 0690519P</t>
+          <t>0692945B, 0690554C</t>
         </is>
       </c>
     </row>
@@ -3132,17 +3132,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EXTERNAT SAINT MICHEL</t>
+          <t>NOTRE DAME DES MINIMES</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SAINT-ETIENNE</t>
+          <t>LYON</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3151,22 +3151,22 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1287</v>
+        <v>1270</v>
       </c>
       <c r="G16" t="n">
-        <v>739</v>
+        <v>641</v>
       </c>
       <c r="H16" t="n">
-        <v>548</v>
+        <v>629</v>
       </c>
       <c r="I16" t="n">
-        <v>7722</v>
+        <v>7620</v>
       </c>
       <c r="J16" t="n">
-        <v>23166</v>
+        <v>22860</v>
       </c>
       <c r="K16" t="n">
-        <v>49.5</v>
+        <v>4.4</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -3175,16 +3175,16 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>11100</v>
+        <v>12382</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>https://www.saint-michel-enseignement.com/</t>
+          <t>https://www.lesminimes-lyon.org/college/presentation/</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>0421804H, 0421021G</t>
+          <t>0692936S, 0690519P</t>
         </is>
       </c>
     </row>
@@ -3194,17 +3194,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ASSOMPTION BELLEVUE</t>
+          <t>EXTERNAT SAINT MICHEL</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LA MULATIERE</t>
+          <t>SAINT-ETIENNE</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -3213,22 +3213,22 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1107</v>
+        <v>1287</v>
       </c>
       <c r="G17" t="n">
-        <v>480</v>
+        <v>739</v>
       </c>
       <c r="H17" t="n">
-        <v>627</v>
+        <v>548</v>
       </c>
       <c r="I17" t="n">
-        <v>6642</v>
+        <v>7722</v>
       </c>
       <c r="J17" t="n">
-        <v>19926</v>
+        <v>23166</v>
       </c>
       <c r="K17" t="n">
-        <v>2.9</v>
+        <v>49.5</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
@@ -3237,16 +3237,16 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>10793</v>
+        <v>11100</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>https://www.assomption-lyon.org/</t>
+          <t>https://www.saint-michel-enseignement.com/</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0692923C, 0690539L</t>
+          <t>0421804H, 0421021G</t>
         </is>
       </c>
     </row>
@@ -3256,17 +3256,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SAINT PAUL</t>
+          <t>ASSOMPTION BELLEVUE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SAINT-ETIENNE</t>
+          <t>LA MULATIERE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -3275,22 +3275,22 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1187</v>
+        <v>1107</v>
       </c>
       <c r="G18" t="n">
-        <v>673</v>
+        <v>480</v>
       </c>
       <c r="H18" t="n">
-        <v>514</v>
+        <v>627</v>
       </c>
       <c r="I18" t="n">
-        <v>7122</v>
+        <v>6642</v>
       </c>
       <c r="J18" t="n">
-        <v>21366</v>
+        <v>19926</v>
       </c>
       <c r="K18" t="n">
-        <v>49.6</v>
+        <v>2.9</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -3299,16 +3299,16 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>10238</v>
+        <v>10793</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>https://www.institutionsaintpaul.org</t>
+          <t>https://www.assomption-lyon.org/</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>0421801E, 0421035X</t>
+          <t>0692923C, 0690539L</t>
         </is>
       </c>
     </row>
@@ -3318,17 +3318,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SAINT PIERRE</t>
+          <t>SAINT PAUL</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BOURG-EN-BRESSE</t>
+          <t>SAINT-ETIENNE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -3337,22 +3337,22 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1246</v>
+        <v>1187</v>
       </c>
       <c r="G19" t="n">
-        <v>807</v>
+        <v>673</v>
       </c>
       <c r="H19" t="n">
-        <v>439</v>
+        <v>514</v>
       </c>
       <c r="I19" t="n">
-        <v>7476</v>
+        <v>7122</v>
       </c>
       <c r="J19" t="n">
-        <v>22428</v>
+        <v>21366</v>
       </c>
       <c r="K19" t="n">
-        <v>58.4</v>
+        <v>49.6</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>9345</v>
+        <v>10238</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>https://www.college-saintpierre.eu/</t>
+          <t>https://www.institutionsaintpaul.org</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0010082J, 0010070W</t>
+          <t>0421801E, 0421035X</t>
         </is>
       </c>
     </row>
@@ -3380,17 +3380,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CHAMPAGNAT</t>
+          <t>SAINT PIERRE</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SAINT-SYMPHORIEN-SUR-COISE</t>
+          <t>BOURG-EN-BRESSE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -3399,22 +3399,22 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1005</v>
+        <v>1246</v>
       </c>
       <c r="G20" t="n">
-        <v>430</v>
+        <v>807</v>
       </c>
       <c r="H20" t="n">
-        <v>575</v>
+        <v>439</v>
       </c>
       <c r="I20" t="n">
-        <v>6030</v>
+        <v>7476</v>
       </c>
       <c r="J20" t="n">
-        <v>18090</v>
+        <v>22428</v>
       </c>
       <c r="K20" t="n">
-        <v>33.2</v>
+        <v>58.4</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -3423,16 +3423,16 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>8668</v>
+        <v>9345</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>http://www.champagnat-stsymphorien.eu/index.php</t>
+          <t>https://www.college-saintpierre.eu/</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0692925E, 0691654Y</t>
+          <t>0010082J, 0010070W</t>
         </is>
       </c>
     </row>
@@ -3442,12 +3442,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SAINT CHARLES</t>
+          <t>CHAMPAGNAT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>RILLIEUX-LA-PAPE</t>
+          <t>SAINT-SYMPHORIEN-SUR-COISE</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -3461,22 +3461,22 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>864</v>
+        <v>1005</v>
       </c>
       <c r="G21" t="n">
-        <v>628</v>
+        <v>430</v>
       </c>
       <c r="H21" t="n">
-        <v>236</v>
+        <v>575</v>
       </c>
       <c r="I21" t="n">
-        <v>5184</v>
+        <v>6030</v>
       </c>
       <c r="J21" t="n">
-        <v>15552</v>
+        <v>18090</v>
       </c>
       <c r="K21" t="n">
-        <v>8.9</v>
+        <v>33.2</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -3485,16 +3485,16 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>8424</v>
+        <v>8668</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>https://st-charles.eu/</t>
+          <t>http://www.champagnat-stsymphorien.eu/index.php</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>0691680B, 0691651V, 0694197M</t>
+          <t>0692925E, 0691654Y</t>
         </is>
       </c>
     </row>
@@ -3504,17 +3504,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SAINT PAUL</t>
+          <t>SAINT CHARLES</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ROANNE</t>
+          <t>RILLIEUX-LA-PAPE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -3523,22 +3523,22 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>927</v>
+        <v>864</v>
       </c>
       <c r="G22" t="n">
-        <v>657</v>
+        <v>628</v>
       </c>
       <c r="H22" t="n">
-        <v>270</v>
+        <v>236</v>
       </c>
       <c r="I22" t="n">
-        <v>5562</v>
+        <v>5184</v>
       </c>
       <c r="J22" t="n">
-        <v>16686</v>
+        <v>15552</v>
       </c>
       <c r="K22" t="n">
-        <v>68</v>
+        <v>8.9</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -3547,16 +3547,16 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>6952</v>
+        <v>8424</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>https://saint-paul-roanne.cybercolleges42.fr/</t>
+          <t>https://st-charles.eu/</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>0421797A, 0421023J</t>
+          <t>0691680B, 0691651V, 0694197M</t>
         </is>
       </c>
     </row>
@@ -3566,12 +3566,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TEZENAS DU MONTCEL</t>
+          <t>SAINT PAUL</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SAINT-ETIENNE</t>
+          <t>ROANNE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3585,22 +3585,22 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>803</v>
+        <v>927</v>
       </c>
       <c r="G23" t="n">
-        <v>495</v>
+        <v>657</v>
       </c>
       <c r="H23" t="n">
-        <v>308</v>
+        <v>270</v>
       </c>
       <c r="I23" t="n">
-        <v>4818</v>
+        <v>5562</v>
       </c>
       <c r="J23" t="n">
-        <v>14454</v>
+        <v>16686</v>
       </c>
       <c r="K23" t="n">
-        <v>49.1</v>
+        <v>68</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -3609,16 +3609,16 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>6926</v>
+        <v>6952</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>https://tezenas.org</t>
+          <t>https://saint-paul-roanne.cybercolleges42.fr/</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>0421741P, 0421742R, 0420979L</t>
+          <t>0421797A, 0421023J</t>
         </is>
       </c>
     </row>
@@ -3628,17 +3628,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SAINT JOSEPH</t>
+          <t>TEZENAS DU MONTCEL</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SAINT-DIDIER-SUR-CHALARONNE</t>
+          <t>SAINT-ETIENNE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -3647,22 +3647,22 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>777</v>
+        <v>803</v>
       </c>
       <c r="G24" t="n">
-        <v>557</v>
+        <v>495</v>
       </c>
       <c r="H24" t="n">
-        <v>220</v>
+        <v>308</v>
       </c>
       <c r="I24" t="n">
-        <v>4662</v>
+        <v>4818</v>
       </c>
       <c r="J24" t="n">
-        <v>13986</v>
+        <v>14454</v>
       </c>
       <c r="K24" t="n">
-        <v>47.8</v>
+        <v>49.1</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -3671,16 +3671,16 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>6702</v>
+        <v>6926</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>http://www.st-joseph01.fr/</t>
+          <t>https://tezenas.org</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>0010095Y, 0011431A</t>
+          <t>0421741P, 0421742R, 0420979L</t>
         </is>
       </c>
     </row>
@@ -3690,59 +3690,59 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PIERRE TERMIER-SITE MONPLAISIR</t>
+          <t>SAINT JOSEPH</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LYON</t>
+          <t>SAINT-DIDIER-SUR-CHALARONNE</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Collège</t>
+          <t>Collège + Lycée GT</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>849</v>
+        <v>777</v>
       </c>
       <c r="G25" t="n">
-        <v>849</v>
+        <v>557</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="I25" t="n">
-        <v>5094</v>
+        <v>4662</v>
       </c>
       <c r="J25" t="n">
-        <v>15282</v>
+        <v>13986</v>
       </c>
       <c r="K25" t="n">
-        <v>2.4</v>
+        <v>47.8</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>6622</v>
+        <v>6702</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>http://www.etablissement-pierretermier.com</t>
+          <t>http://www.st-joseph01.fr/</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>0692940W</t>
+          <t>0010095Y, 0011431A</t>
         </is>
       </c>
     </row>
@@ -3752,59 +3752,59 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SAINT JOSEPH</t>
+          <t>PIERRE TERMIER-SITE MONPLAISIR</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MIRIBEL</t>
+          <t>LYON</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Collège + Lycée GT</t>
+          <t>Collège</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>599</v>
+        <v>849</v>
       </c>
       <c r="G26" t="n">
-        <v>336</v>
+        <v>849</v>
       </c>
       <c r="H26" t="n">
-        <v>263</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>3594</v>
+        <v>5094</v>
       </c>
       <c r="J26" t="n">
-        <v>10782</v>
+        <v>15282</v>
       </c>
       <c r="K26" t="n">
-        <v>11.9</v>
+        <v>2.4</v>
       </c>
       <c r="L26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>5840</v>
+        <v>6622</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>https://www.saintjoseph01.fr/</t>
+          <t>http://www.etablissement-pierretermier.com</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>0011151W, 0010075B</t>
+          <t>0692940W</t>
         </is>
       </c>
     </row>
@@ -3814,12 +3814,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>NOTRE DAME DE MONGRE</t>
+          <t>NOTRE DAME DE BEL AIR</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>VILLEFRANCHE-SUR-SAONE</t>
+          <t>TARARE</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3833,22 +3833,22 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1789</v>
+        <v>973</v>
       </c>
       <c r="G27" t="n">
-        <v>1115</v>
+        <v>421</v>
       </c>
       <c r="H27" t="n">
-        <v>674</v>
+        <v>552</v>
       </c>
       <c r="I27" t="n">
-        <v>10734</v>
+        <v>5838</v>
       </c>
       <c r="J27" t="n">
-        <v>32202</v>
+        <v>17514</v>
       </c>
       <c r="K27" t="n">
-        <v>28.8</v>
+        <v>35.5</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -3857,16 +3857,16 @@
         <v>1</v>
       </c>
       <c r="N27" t="n">
-        <v>15430</v>
+        <v>8392</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>https://www.mongre.org/</t>
+          <t>https://www.csnd.fr/colleges/college-notre-dame-de-bel-air-tarare/</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>0692944A, 0690552A</t>
+          <t>0690618X, 0693267B</t>
         </is>
       </c>
     </row>
@@ -3876,17 +3876,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>NOTRE DAME DE BEL AIR</t>
+          <t>SAINT JOSEPH</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>TARARE</t>
+          <t>MIRIBEL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3895,40 +3895,40 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>973</v>
+        <v>599</v>
       </c>
       <c r="G28" t="n">
-        <v>421</v>
+        <v>336</v>
       </c>
       <c r="H28" t="n">
-        <v>552</v>
+        <v>263</v>
       </c>
       <c r="I28" t="n">
-        <v>5838</v>
+        <v>3594</v>
       </c>
       <c r="J28" t="n">
-        <v>17514</v>
+        <v>10782</v>
       </c>
       <c r="K28" t="n">
-        <v>35.5</v>
+        <v>11.9</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>8392</v>
+        <v>5840</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>https://www.csnd.fr/colleges/college-notre-dame-de-bel-air-tarare/</t>
+          <t>https://www.saintjoseph01.fr/</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>0690618X, 0693267B</t>
+          <t>0011151W, 0010075B</t>
         </is>
       </c>
     </row>
@@ -10047,7 +10047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10156,12 +10156,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NOTRE DAME DE MONGRE</t>
+          <t>NOTRE DAME DE BEL AIR</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>VILLEFRANCHE-SUR-SAONE</t>
+          <t>TARARE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -10175,22 +10175,22 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1789</v>
+        <v>973</v>
       </c>
       <c r="G2" t="n">
-        <v>1115</v>
+        <v>421</v>
       </c>
       <c r="H2" t="n">
-        <v>674</v>
+        <v>552</v>
       </c>
       <c r="I2" t="n">
-        <v>10734</v>
+        <v>5838</v>
       </c>
       <c r="J2" t="n">
-        <v>32202</v>
+        <v>17514</v>
       </c>
       <c r="K2" t="n">
-        <v>28.8</v>
+        <v>35.5</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -10199,16 +10199,16 @@
         <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>15430</v>
+        <v>8392</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>https://www.mongre.org/</t>
+          <t>https://www.csnd.fr/colleges/college-notre-dame-de-bel-air-tarare/</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0692944A, 0690552A</t>
+          <t>0690618X, 0693267B</t>
         </is>
       </c>
     </row>
@@ -10218,12 +10218,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NOTRE DAME DE BEL AIR</t>
+          <t>NOTRE DAME</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TARARE</t>
+          <t>VILLEFRANCHE-SUR-SAONE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -10237,22 +10237,22 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>973</v>
+        <v>401</v>
       </c>
       <c r="G3" t="n">
-        <v>421</v>
+        <v>59</v>
       </c>
       <c r="H3" t="n">
-        <v>552</v>
+        <v>342</v>
       </c>
       <c r="I3" t="n">
-        <v>5838</v>
+        <v>2406</v>
       </c>
       <c r="J3" t="n">
-        <v>17514</v>
+        <v>7218</v>
       </c>
       <c r="K3" t="n">
-        <v>35.5</v>
+        <v>28.3</v>
       </c>
       <c r="L3" t="n">
         <v>1</v>
@@ -10261,16 +10261,16 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>8392</v>
+        <v>3459</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>https://www.csnd.fr/colleges/college-notre-dame-de-bel-air-tarare/</t>
+          <t>https://www.csnd.fr</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>0690618X, 0693267B</t>
+          <t>0693375U, 0690553B</t>
         </is>
       </c>
     </row>
@@ -10285,7 +10285,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>VILLEFRANCHE-SUR-SAONE</t>
+          <t>BELLEVILLE-EN-BEAUJOLAIS</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -10295,44 +10295,39 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Collège + Lycée GT</t>
+          <t>Collège</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>401</v>
+        <v>438</v>
       </c>
       <c r="G4" t="n">
-        <v>59</v>
+        <v>438</v>
       </c>
       <c r="H4" t="n">
-        <v>342</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>2406</v>
+        <v>2628</v>
       </c>
       <c r="J4" t="n">
-        <v>7218</v>
+        <v>7884</v>
       </c>
       <c r="K4" t="n">
-        <v>28.3</v>
+        <v>42.1</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
         <v>1</v>
       </c>
       <c r="N4" t="n">
-        <v>3459</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>https://www.csnd.fr</t>
-        </is>
+        <v>3022</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0693375U, 0690553B</t>
+          <t>0694279B</t>
         </is>
       </c>
     </row>
@@ -10342,12 +10337,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NOTRE DAME</t>
+          <t>NOTRE DAME DU MAS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BELLEVILLE-EN-BEAUJOLAIS</t>
+          <t>VAL D'OINGT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -10361,22 +10356,22 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>438</v>
+        <v>363</v>
       </c>
       <c r="G5" t="n">
-        <v>438</v>
+        <v>363</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>2628</v>
+        <v>2178</v>
       </c>
       <c r="J5" t="n">
-        <v>7884</v>
+        <v>6534</v>
       </c>
       <c r="K5" t="n">
-        <v>42.1</v>
+        <v>28.1</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -10385,11 +10380,16 @@
         <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>3022</v>
+        <v>2505</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>https://www.csnd.fr/scolarite-college/college-notre-dame-du-mas/</t>
+        </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>0694279B</t>
+          <t>0690580F</t>
         </is>
       </c>
     </row>
@@ -10399,12 +10399,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NOTRE DAME DU MAS</t>
+          <t>NOTRE DAME</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>VAL D'OINGT</t>
+          <t>CLAVEISOLLES</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -10418,22 +10418,22 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>363</v>
+        <v>66</v>
       </c>
       <c r="G6" t="n">
-        <v>363</v>
+        <v>66</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>2178</v>
+        <v>396</v>
       </c>
       <c r="J6" t="n">
-        <v>6534</v>
+        <v>1188</v>
       </c>
       <c r="K6" t="n">
-        <v>28.1</v>
+        <v>47.8</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -10442,83 +10442,21 @@
         <v>1</v>
       </c>
       <c r="N6" t="n">
-        <v>2505</v>
+        <v>455</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>https://www.csnd.fr/scolarite-college/college-notre-dame-du-mas/</t>
+          <t>https://www.csnd.fr/colleges/college-notre-dame-claveisolles/</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0690580F</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>0</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>NOTRE DAME</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CLAVEISOLLES</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>69</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Collège</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>66</v>
-      </c>
-      <c r="G7" t="n">
-        <v>66</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>396</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1188</v>
-      </c>
-      <c r="K7" t="n">
-        <v>47.8</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" t="n">
-        <v>455</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>https://www.csnd.fr/colleges/college-notre-dame-claveisolles/</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
           <t>0690585L</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P7"/>
+  <autoFilter ref="A1:P6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>